<commit_message>
Veri doğrulama kuralları düzenlendi
</commit_message>
<xml_diff>
--- a/Public/assets/downloads/Hoca listesi.xlsx
+++ b/Public/assets/downloads/Hoca listesi.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sayfa2" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Samet ATABAŞ</author>
   </authors>
@@ -36,13 +37,34 @@
           <t xml:space="preserve">Üniversite mail adresi</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>23</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>34</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>17</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
   <si>
     <t xml:space="preserve">Mail</t>
   </si>
@@ -63,6 +85,108 @@
   </si>
   <si>
     <t xml:space="preserve">Programı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bölümler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programlar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilgisayar Teknolojileri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilgisayar Programcılığı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Akademisyen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prof. Dr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elektrik ve Enerji</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web Tasarımı ve Kodlama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bölüm Başkanı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doç. Dr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muhasebe Ve Vergi Uygulamaları</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elektrik Üretim İletim ve Dağıtım</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Müdür Yardımcısı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. Öğr. Üyesi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yönetim ve Organizasyon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alternatif Enerji Kaynakları Teknolojisi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Müdür</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Öğr. Gör.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finans - Bankacılık ve Sigortacılık</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geleneksel El Sanatları</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Araş. Gör.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Sanatları</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kuyumculuk ve Takı Tasarımı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seyahat - Turizm ve Eğlence Hizmetleri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bankacılık ve Sigortacılık Programı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ulaştırma Hizmetleri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maliye</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mimarlık Ve Şehir Planlama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Turizm ve Seyahat Hizmetleri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">İşletme Yönetimi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sağlık Kurumları İşletmeciliği</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posta Hizmetleri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ulaştırma ve Trafik Hizmetleri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tapu ve Kadastro</t>
   </si>
 </sst>
 </file>
@@ -156,7 +280,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -175,6 +299,14 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -197,37 +329,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -301,7 +433,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G41"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.27"/>
@@ -684,25 +816,21 @@
       <c r="E41" s="4"/>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2 E4:E41" type="list">
-      <formula1>"Akademisyen,Bölüm Başkanı,Müdür Yardımcısı,Müdür"</formula1>
+  <dataValidations count="4">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F1001" type="list">
+      <formula1>Sayfa2!$A$2:$A$100</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B41" type="list">
-      <formula1>"Prof. Dr.,Doç. Dr.,Dr. Öğr. Üyesi,Öğr. Gör.,Araş. Gör."</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G1001" type="list">
+      <formula1>Sayfa2!$B$2:$B$100</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G38" type="list">
-      <formula1>"Bilgisayar Programcılığı,Web Tasarımı ve Kodlama,Elektrik Üretim İletim ve Dağıtım,Alternatif Enerji Kaynakları Teknolojisi,Geleneksel El Sanatları,Kuyumculuk ve Takı Tasarımı,Bankacılık ve Sigortacılık Programı,Maliye,Muhasebe Ve Vergi Uygulamaları,Turiz"</formula1>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E1001" type="list">
+      <formula1>Sayfa2!$C$2:$C$100</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F38" type="list">
-      <formula1>"Bilgisayar Teknolojileri,Elektrik ve Enerji,Muhasebe ve Vergi Uygulamaları,Yönetim ve Organizasyon,Finans - Bankacılık ve Sigortacılık,El Sanatları,Seyahat - Turizm ve Eğlence Hizmetleri,Ulaştırma Hizmetleri,Mimarlık Ve Şehir Planlama"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E3" type="list">
-      <formula1>"Akademisyen,Bölüm Başkanı,Müdür Yardımcısı,Müdür"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B1001" type="list">
+      <formula1>Sayfa2!$D$2:$D$100</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -715,4 +843,178 @@
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="33.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.43"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1"/>
+      <c r="B11" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1"/>
+      <c r="B12" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1"/>
+      <c r="B13" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1"/>
+      <c r="B14" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1"/>
+      <c r="B15" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1"/>
+      <c r="B16" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Sayfa &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor: Gate authorize metodu DTO desteği ile güncellendi ve tüm create policy kontrolleri objelere uyarlandı
</commit_message>
<xml_diff>
--- a/Public/assets/downloads/Hoca listesi.xlsx
+++ b/Public/assets/downloads/Hoca listesi.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" state="visible" r:id="rId3"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="79">
   <si>
     <t xml:space="preserve">Mail</t>
   </si>
@@ -81,16 +81,13 @@
     <t xml:space="preserve">Görevi</t>
   </si>
   <si>
-    <t xml:space="preserve">Bölümü</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Programı</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bölümler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Programlar</t>
+    <t xml:space="preserve">Fakülte / MYO / Enstitü</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bölümü / Ana Bilim Dalı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programı / Bilim Dalı</t>
   </si>
   <si>
     <t xml:space="preserve">Bilgisayar Teknolojileri</t>
@@ -117,6 +114,9 @@
     <t xml:space="preserve">Doç. Dr.</t>
   </si>
   <si>
+    <t xml:space="preserve">Fen Bilimleri Enstitüsü</t>
+  </si>
+  <si>
     <t xml:space="preserve">Muhasebe Ve Vergi Uygulamaları</t>
   </si>
   <si>
@@ -129,6 +129,9 @@
     <t xml:space="preserve">Dr. Öğr. Üyesi</t>
   </si>
   <si>
+    <t xml:space="preserve">Sağlık Bilimleri Enstitüsü</t>
+  </si>
+  <si>
     <t xml:space="preserve">Yönetim ve Organizasyon</t>
   </si>
   <si>
@@ -141,12 +144,18 @@
     <t xml:space="preserve">Öğr. Gör.</t>
   </si>
   <si>
+    <t xml:space="preserve">Sosyal Bilimler Enstitüsü</t>
+  </si>
+  <si>
     <t xml:space="preserve">Finans - Bankacılık ve Sigortacılık</t>
   </si>
   <si>
     <t xml:space="preserve">Geleneksel El Sanatları</t>
   </si>
   <si>
+    <t xml:space="preserve">Sekreter</t>
+  </si>
+  <si>
     <t xml:space="preserve">Araş. Gör.</t>
   </si>
   <si>
@@ -156,37 +165,142 @@
     <t xml:space="preserve">Kuyumculuk ve Takı Tasarımı</t>
   </si>
   <si>
+    <t xml:space="preserve">Araştırma Görevlisi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Denizcilik Fakültesi</t>
+  </si>
+  <si>
     <t xml:space="preserve">Seyahat - Turizm ve Eğlence Hizmetleri</t>
   </si>
   <si>
     <t xml:space="preserve">Bankacılık ve Sigortacılık Programı</t>
   </si>
   <si>
+    <t xml:space="preserve">Diş Hekimliği Fakültesi</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ulaştırma Hizmetleri</t>
   </si>
   <si>
     <t xml:space="preserve">Maliye</t>
   </si>
   <si>
+    <t xml:space="preserve">Eğitim Fakültesi</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mimarlık Ve Şehir Planlama</t>
   </si>
   <si>
+    <t xml:space="preserve">Fen Edebiyat Fakültesi</t>
+  </si>
+  <si>
     <t xml:space="preserve">Turizm ve Seyahat Hizmetleri</t>
   </si>
   <si>
+    <t xml:space="preserve">Güzel Sanatlar Fakültesi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Halkla İlişkiler ve Tanıtım</t>
+  </si>
+  <si>
     <t xml:space="preserve">İşletme Yönetimi</t>
   </si>
   <si>
+    <t xml:space="preserve">İktisadi ve İdari Bilimler Fakültesi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gazetecilik</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sağlık Kurumları İşletmeciliği</t>
   </si>
   <si>
+    <t xml:space="preserve">İlahiyat Fakültesi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Radyo, Televizyon ve Sinema</t>
+  </si>
+  <si>
     <t xml:space="preserve">Posta Hizmetleri</t>
   </si>
   <si>
+    <t xml:space="preserve">Mühendislik Fakültesi</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ulaştırma ve Trafik Hizmetleri</t>
   </si>
   <si>
+    <t xml:space="preserve">Sağlık Bilimleri Fakültesi</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tapu ve Kadastro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spor Bilimleri Fakültesi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tıp Fakültesi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tirebolu İletişim Fakültesi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Turizm Fakültesi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulancak Kadir Karabaş Uygulamalı Bilimler Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Devlet Konservatuvarı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Görele Uygulamalı Bilimler Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sivil Havacılık Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Şebinkarahisar Uygulamalı Bilimler Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yabancı Diller Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alucra Turan Bulutçu Meslek Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulancak Meslek Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dereli Meslek Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espiye Meslek Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eynesil Kamil Nalbant Meslek Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giresun Meslek Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keşap Meslek Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piraziz Meslek Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sağlık Hizmetleri Meslek Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Şebinkarahisar Meslek Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Şebinkarahisar Sağlık Hizmetleri Meslek Yüksekokulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tirebolu Mehmet Bayrak Meslek Yüksekokulu</t>
   </si>
 </sst>
 </file>
@@ -196,7 +310,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -236,6 +350,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -280,7 +401,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -301,11 +422,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -432,7 +557,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.37"/>
@@ -440,8 +565,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.97"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="33.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="32.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="38.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="33.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="32.35"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -465,6 +591,9 @@
       </c>
       <c r="G1" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -475,6 +604,7 @@
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3"/>
@@ -484,6 +614,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3"/>
@@ -493,6 +624,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3"/>
@@ -502,6 +634,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3"/>
@@ -511,6 +644,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3"/>
@@ -520,6 +654,7 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3"/>
@@ -529,6 +664,7 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3"/>
@@ -538,6 +674,7 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3"/>
@@ -547,6 +684,7 @@
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3"/>
@@ -556,6 +694,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3"/>
@@ -565,6 +704,7 @@
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3"/>
@@ -574,6 +714,7 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3"/>
@@ -583,6 +724,7 @@
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3"/>
@@ -592,6 +734,7 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3"/>
@@ -601,6 +744,7 @@
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3"/>
@@ -610,6 +754,7 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3"/>
@@ -619,6 +764,7 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3"/>
@@ -628,6 +774,7 @@
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3"/>
@@ -637,6 +784,7 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3"/>
@@ -646,6 +794,7 @@
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3"/>
@@ -655,6 +804,7 @@
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3"/>
@@ -664,6 +814,7 @@
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3"/>
@@ -673,6 +824,7 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3"/>
@@ -682,6 +834,7 @@
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3"/>
@@ -691,6 +844,7 @@
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3"/>
@@ -700,6 +854,7 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3"/>
@@ -709,6 +864,7 @@
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3"/>
@@ -718,6 +874,7 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3"/>
@@ -727,6 +884,7 @@
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3"/>
@@ -736,6 +894,7 @@
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3"/>
@@ -745,6 +904,7 @@
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3"/>
@@ -754,6 +914,7 @@
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3"/>
@@ -763,6 +924,7 @@
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3"/>
@@ -772,6 +934,7 @@
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3"/>
@@ -781,6 +944,7 @@
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
+      <c r="H36" s="4"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3"/>
@@ -790,6 +954,7 @@
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
+      <c r="H37" s="4"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3"/>
@@ -799,29 +964,33 @@
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3"/>
       <c r="B39" s="4"/>
       <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3"/>
       <c r="B40" s="4"/>
       <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3"/>
       <c r="B41" s="4"/>
       <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F1001" type="list">
+  <dataValidations count="5">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G1001" type="list">
       <formula1>Sayfa2!$A$2:$A$100</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G1001" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H1001" type="list">
       <formula1>Sayfa2!$B$2:$B$100</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -831,6 +1000,10 @@
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B1001" type="list">
       <formula1>Sayfa2!$D$2:$D$100</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F1001" type="list">
+      <formula1>Sayfa2!$E$2:$E$100</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -850,165 +1023,375 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="33.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="33.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21.98"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+      <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="E2" s="6"/>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="B3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="E3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="E4" s="7" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>21</v>
+      <c r="A5" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="D5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>25</v>
+      <c r="A6" s="5" t="s">
+        <v>27</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>27</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>28</v>
+      <c r="A7" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>30</v>
+      <c r="A8" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>32</v>
+      <c r="A9" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>33</v>
+        <v>39</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>34</v>
+      <c r="A10" s="5" t="s">
+        <v>41</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="E10" s="7" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1"/>
-      <c r="B11" s="6" t="s">
-        <v>35</v>
+      <c r="B11" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1"/>
-      <c r="B12" s="6" t="s">
-        <v>36</v>
+      <c r="A12" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1"/>
-      <c r="B13" s="6" t="s">
-        <v>37</v>
+      <c r="A13" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1"/>
-      <c r="B14" s="6" t="s">
-        <v>38</v>
+      <c r="A14" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1"/>
-      <c r="B15" s="6" t="s">
-        <v>39</v>
+      <c r="B15" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1"/>
-      <c r="B16" s="6" t="s">
-        <v>40</v>
+      <c r="B16" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E17" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E20" s="6"/>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E21" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E22" s="7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E23" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E24" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E25" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E26" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E27" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E28" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E29" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E30" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E31" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E32" s="7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E33" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E34" s="7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E35" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E36" s="7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E37" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E38" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E39" s="7" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E3" r:id="rId1" display="Fen Bilimleri Enstitüsü"/>
+    <hyperlink ref="E4" r:id="rId2" display="Sağlık Bilimleri Enstitüsü"/>
+    <hyperlink ref="E5" r:id="rId3" display="Sosyal Bilimler Enstitüsü"/>
+    <hyperlink ref="E7" r:id="rId4" display="Denizcilik Fakültesi"/>
+    <hyperlink ref="E8" r:id="rId5" display="Diş Hekimliği Fakültesi"/>
+    <hyperlink ref="E9" r:id="rId6" display="Eğitim Fakültesi"/>
+    <hyperlink ref="E10" r:id="rId7" display="Fen Edebiyat Fakültesi"/>
+    <hyperlink ref="E11" r:id="rId8" display="Güzel Sanatlar Fakültesi"/>
+    <hyperlink ref="E12" r:id="rId9" display="İktisadi ve İdari Bilimler Fakültesi"/>
+    <hyperlink ref="E13" r:id="rId10" display="İlahiyat Fakültesi"/>
+    <hyperlink ref="E14" r:id="rId11" display="Mühendislik Fakültesi"/>
+    <hyperlink ref="E15" r:id="rId12" display="Sağlık Bilimleri Fakültesi"/>
+    <hyperlink ref="E16" r:id="rId13" display="Spor Bilimleri Fakültesi"/>
+    <hyperlink ref="E17" r:id="rId14" display="Tıp Fakültesi"/>
+    <hyperlink ref="E18" r:id="rId15" display="Tirebolu İletişim Fakültesi"/>
+    <hyperlink ref="E19" r:id="rId16" display="Turizm Fakültesi"/>
+    <hyperlink ref="E21" r:id="rId17" display="Bulancak Kadir Karabaş Uygulamalı Bilimler Yüksekokulu"/>
+    <hyperlink ref="E22" r:id="rId18" display="Devlet Konservatuvarı"/>
+    <hyperlink ref="E23" r:id="rId19" display="Görele Uygulamalı Bilimler Yüksekokulu"/>
+    <hyperlink ref="E24" r:id="rId20" display="Sivil Havacılık Yüksekokulu"/>
+    <hyperlink ref="E25" r:id="rId21" display="Şebinkarahisar Uygulamalı Bilimler Yüksekokulu"/>
+    <hyperlink ref="E26" r:id="rId22" display="Yabancı Diller Yüksekokulu"/>
+    <hyperlink ref="E28" r:id="rId23" display="Alucra Turan Bulutçu Meslek Yüksekokulu"/>
+    <hyperlink ref="E29" r:id="rId24" display="Bulancak Meslek Yüksekokulu"/>
+    <hyperlink ref="E30" r:id="rId25" display="Dereli Meslek Yüksekokulu"/>
+    <hyperlink ref="E31" r:id="rId26" display="Espiye Meslek Yüksekokulu"/>
+    <hyperlink ref="E32" r:id="rId27" display="Eynesil Kamil Nalbant Meslek Yüksekokulu"/>
+    <hyperlink ref="E33" r:id="rId28" display="Giresun Meslek Yüksekokulu"/>
+    <hyperlink ref="E34" r:id="rId29" display="Keşap Meslek Yüksekokulu"/>
+    <hyperlink ref="E35" r:id="rId30" display="Piraziz Meslek Yüksekokulu"/>
+    <hyperlink ref="E36" r:id="rId31" display="Sağlık Hizmetleri Meslek Yüksekokulu"/>
+    <hyperlink ref="E37" r:id="rId32" display="Şebinkarahisar Meslek Yüksekokulu"/>
+    <hyperlink ref="E38" r:id="rId33" display="Şebinkarahisar Sağlık Hizmetleri Meslek Yüksekokulu"/>
+    <hyperlink ref="E39" r:id="rId34" display="Tirebolu Mehmet Bayrak Meslek Yüksekokulu"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
hoca içe aktarma excel i ve işlemleri düzenlendi #83
</commit_message>
<xml_diff>
--- a/Public/assets/downloads/Hoca listesi.xlsx
+++ b/Public/assets/downloads/Hoca listesi.xlsx
@@ -310,7 +310,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -350,13 +350,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -401,7 +394,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -426,11 +419,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1030,7 +1019,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="33.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.98"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1063,7 +1052,7 @@
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -1078,7 +1067,7 @@
       <c r="D3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1095,7 +1084,7 @@
       <c r="D4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="6" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1112,7 +1101,7 @@
       <c r="D5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="6" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1129,7 +1118,7 @@
       <c r="D6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="6"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
@@ -1141,7 +1130,7 @@
       <c r="C7" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="6" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1152,7 +1141,7 @@
       <c r="B8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1163,7 +1152,7 @@
       <c r="B9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="6" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1174,7 +1163,7 @@
       <c r="B10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="6" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1182,7 +1171,7 @@
       <c r="B11" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="6" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1193,7 +1182,7 @@
       <c r="B12" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="6" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1204,7 +1193,7 @@
       <c r="B13" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="6" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1215,7 +1204,7 @@
       <c r="B14" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="6" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1223,7 +1212,7 @@
       <c r="B15" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="6" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1231,12 +1220,12 @@
       <c r="B16" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="6" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1244,7 +1233,7 @@
       <c r="B18" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="6" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1252,7 +1241,7 @@
       <c r="B19" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="6" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1260,98 +1249,98 @@
       <c r="B20" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="6" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="6" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="6" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="6" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E26" s="7" t="s">
+      <c r="E26" s="6" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E27" s="6"/>
+      <c r="E27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E28" s="7" t="s">
+      <c r="E28" s="6" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E29" s="7" t="s">
+      <c r="E29" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E30" s="7" t="s">
+      <c r="E30" s="6" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E31" s="7" t="s">
+      <c r="E31" s="6" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E32" s="7" t="s">
+      <c r="E32" s="6" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E33" s="7" t="s">
+      <c r="E33" s="6" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E34" s="7" t="s">
+      <c r="E34" s="6" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E35" s="7" t="s">
+      <c r="E35" s="6" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E36" s="7" t="s">
+      <c r="E36" s="6" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E37" s="7" t="s">
+      <c r="E37" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E38" s="7" t="s">
+      <c r="E38" s="6" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E39" s="7" t="s">
+      <c r="E39" s="6" t="s">
         <v>78</v>
       </c>
     </row>

</xml_diff>